<commit_message>
Link chemical registrations to existing library materials and restore shared categories
</commit_message>
<xml_diff>
--- a/pheno-lab/src/infrastructure/chemistry/assets/sam-upload-template.xlsx
+++ b/pheno-lab/src/infrastructure/chemistry/assets/sam-upload-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SAM Materials" sheetId="1" r:id="Rffa0d85120794ed4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Rdc0515c560024a1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SAM Materials" sheetId="1" r:id="R7f1332c79d684daf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R743d80b9df3d4010"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -758,10 +758,10 @@
     </x:row>
     <x:row r="2" ht="54" customHeight="1">
       <x:c r="A2" s="13" t="str">
-        <x:v>Pheno Chemicals SAM upload</x:v>
+        <x:v>Pheno Chemicals material upload</x:v>
       </x:c>
       <x:c r="B2" s="13" t="str">
-        <x:v>Pheno Chemicals SAM 批量录入</x:v>
+        <x:v>Pheno Chemicals 材料批量录入</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="54" customHeight="1">
@@ -774,18 +774,18 @@
     </x:row>
     <x:row r="4" ht="54" customHeight="1">
       <x:c r="A4" s="10" t="str">
-        <x:v>Start at row 2. Enter one new molecule name and its SMILES per row.</x:v>
+        <x:v>Start at row 2. Enter one molecule name and its SMILES per row.</x:v>
       </x:c>
       <x:c r="B4" s="10" t="str">
-        <x:v>从第 2 行开始，每行填写一个新分子名称及其 SMILES。</x:v>
+        <x:v>从第 2 行开始，每行填写一个分子名称及其 SMILES。</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="54" customHeight="1">
       <x:c r="A5" s="10" t="str">
-        <x:v>All entries are SAM materials. Use plain text; do not enter formulas.</x:v>
+        <x:v>Choose SAM, Additives, Solvents or a custom category on the upload page. All rows use that category.</x:v>
       </x:c>
       <x:c r="B5" s="10" t="str">
-        <x:v>全部按 SAM 材料保存。请填写纯文本，不要使用 Excel 公式。</x:v>
+        <x:v>在上传页面选择 SAM、添加剂、溶剂或自定义类别，整份文件使用该类别。请填写纯文本，不要使用公式。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="54" customHeight="1">
@@ -822,10 +822,10 @@
     </x:row>
     <x:row r="10" ht="54" customHeight="1">
       <x:c r="A10" s="10" t="str">
-        <x:v>Existing or duplicate names are rejected. Imports add materials without overwriting existing records.</x:v>
+        <x:v>Existing library names link to the same record. Names already in Pheno Chemicals and duplicate file rows are rejected.</x:v>
       </x:c>
       <x:c r="B10" s="10" t="str">
-        <x:v>已有名称或文件内重复名称会被拒绝。导入仅新增材料，不覆盖现有记录。</x:v>
+        <x:v>共享材料库中的已有名称会关联同一记录，不重复创建。已在 Pheno Chemicals 中的名称及文件内重名行会被拒绝。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="54" customHeight="1">

</xml_diff>

<commit_message>
Remove Chemicals upload row quota and batch database operations
</commit_message>
<xml_diff>
--- a/pheno-lab/src/infrastructure/chemistry/assets/sam-upload-template.xlsx
+++ b/pheno-lab/src/infrastructure/chemistry/assets/sam-upload-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SAM Materials" sheetId="1" r:id="R7f1332c79d684daf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R743d80b9df3d4010"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SAM Materials" sheetId="1" r:id="Rdd38541c0928479d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Redc88a0b812e4326"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -790,10 +790,10 @@
     </x:row>
     <x:row r="6" ht="54" customHeight="1">
       <x:c r="A6" s="10" t="str">
-        <x:v>Upload up to 100 materials in one .xlsx file, no larger than 2 MB.</x:v>
+        <x:v>Add more rows as needed; there is no material-row quota. Keep each .xlsx file within 2 MB.</x:v>
       </x:c>
       <x:c r="B6" s="10" t="str">
-        <x:v>每个 .xlsx 文件最多 100 个材料，文件大小不超过 2 MB。</x:v>
+        <x:v>可按需继续添加材料行，不设行数上限；每个 .xlsx 文件不超过 2 MB。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="54" customHeight="1">

</xml_diff>

<commit_message>
Allow editing chemical upload drafts and 5 MB workbooks
</commit_message>
<xml_diff>
--- a/pheno-lab/src/infrastructure/chemistry/assets/sam-upload-template.xlsx
+++ b/pheno-lab/src/infrastructure/chemistry/assets/sam-upload-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SAM Materials" sheetId="1" r:id="Rdd38541c0928479d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Redc88a0b812e4326"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SAM Materials" sheetId="1" r:id="R11dc9ab0d06b42d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R3cd84ca268f24563"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -790,10 +790,10 @@
     </x:row>
     <x:row r="6" ht="54" customHeight="1">
       <x:c r="A6" s="10" t="str">
-        <x:v>Add more rows as needed; there is no material-row quota. Keep each .xlsx file within 2 MB.</x:v>
+        <x:v>Add more rows as needed; there is no material-row quota. Keep each .xlsx file within 5 MB.</x:v>
       </x:c>
       <x:c r="B6" s="10" t="str">
-        <x:v>可按需继续添加材料行，不设行数上限；每个 .xlsx 文件不超过 2 MB。</x:v>
+        <x:v>可按需继续添加材料行，不设行数上限；每个 .xlsx 文件不超过 5 MB。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="54" customHeight="1">
@@ -814,18 +814,18 @@
     </x:row>
     <x:row r="9" ht="54" customHeight="1">
       <x:c r="A9" s="10" t="str">
-        <x:v>Correct reported errors in Excel, upload again, then choose Import materials.</x:v>
+        <x:v>Edit names/SMILES or remove selected rows in the preview. Validate changes, then import the remaining rows.</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>在 Excel 中修正提示的错误后重新上传，再点击导入材料。</x:v>
+        <x:v>可在预览中修改名称和 SMILES，或勾选移除行；验证修改后，再导入剩余材料。</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="54" customHeight="1">
       <x:c r="A10" s="10" t="str">
-        <x:v>Existing library names link to the same record. Names already in Pheno Chemicals and duplicate file rows are rejected.</x:v>
+        <x:v>Existing library names link to the same record. Remove already registered or duplicate rows from the upload, or edit their existing portal records.</x:v>
       </x:c>
       <x:c r="B10" s="10" t="str">
-        <x:v>共享材料库中的已有名称会关联同一记录，不重复创建。已在 Pheno Chemicals 中的名称及文件内重名行会被拒绝。</x:v>
+        <x:v>共享材料库中的已有名称会关联同一记录，不重复创建。可从本次上传移除已登记或重复的行，或在入口编辑其已有记录。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="54" customHeight="1">

</xml_diff>